<commit_message>
Add 5-year projections with growth rates
Revenue grows 10% per year, costs grow 5% per year
</commit_message>
<xml_diff>
--- a/profit_calculator.xlsx
+++ b/profit_calculator.xlsx
@@ -413,37 +413,113 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="B1" t="n">
-        <v>100</v>
+      <c r="A1" t="inlineStr"/>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Costs</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>90</v>
+        <v>100</v>
+      </c>
+      <c r="C2">
+        <f>B2*1.1</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>C2*1.1</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>D2*1.1</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>E2*1.1</f>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Costs</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>90</v>
+      </c>
+      <c r="C3">
+        <f>B3*1.05</f>
+        <v/>
+      </c>
+      <c r="D3">
+        <f>C3*1.05</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>D3*1.05</f>
+        <v/>
+      </c>
+      <c r="F3">
+        <f>E3*1.05</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Profit</t>
         </is>
       </c>
-      <c r="B3">
-        <f>B1-B2</f>
+      <c r="B4">
+        <f>B2-B3</f>
+        <v/>
+      </c>
+      <c r="C4">
+        <f>C2-C3</f>
+        <v/>
+      </c>
+      <c r="D4">
+        <f>D2-D3</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>E2-E3</f>
+        <v/>
+      </c>
+      <c r="F4">
+        <f>F2-F3</f>
         <v/>
       </c>
     </row>

</xml_diff>